<commit_message>
Lists: transliterate Arabic names to English, regenerate all 6 Excel files (+Ahmed Tier A)
</commit_message>
<xml_diff>
--- a/Email_Seniors.xlsx
+++ b/Email_Seniors.xlsx
@@ -427,7 +427,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="41" customWidth="1" min="5" max="5"/>
@@ -1622,12 +1622,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>أحمد</t>
+          <t>Ahmed</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>أبوخزيمة</t>
+          <t>Abou Khezaima</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -12810,12 +12810,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>محمود</t>
+          <t>Mahmoud</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>شعبان</t>
+          <t>Shaaban</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -20097,7 +20097,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Al-Attyat صبا العطيات</t>
+          <t>Al-Attyat</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">

</xml_diff>